<commit_message>
feat: mettre à jour les fichiers Excel de parcours et supprimer les fichiers temporaires
</commit_message>
<xml_diff>
--- a/parcours.xlsx
+++ b/parcours.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Nicolas\kDrive\1- IUT\Mission Maroc\Carte\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D2BFE17-3823-4F3B-A1B8-6538F5A21595}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32307FDB-587C-43C8-AF1B-E1710C4E2B00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{F6E9AC9D-BA70-4E60-AAFF-43E24562E406}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{F6E9AC9D-BA70-4E60-AAFF-43E24562E406}"/>
   </bookViews>
   <sheets>
     <sheet name="Parcours" sheetId="1" r:id="rId1"/>

</xml_diff>